<commit_message>
adding analysis on nutrients and traits
</commit_message>
<xml_diff>
--- a/Summary.xlsx
+++ b/Summary.xlsx
@@ -481,7 +481,7 @@
       <c r="B1" s="1" t="inlineStr"/>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>[C_b]%</t>
+          <t>[C_b]</t>
         </is>
       </c>
       <c r="D1" s="1" t="n"/>
@@ -518,7 +518,7 @@
       <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>[C]%</t>
+          <t>[C]</t>
         </is>
       </c>
       <c r="Q1" s="1" t="n"/>
@@ -2117,8 +2117,12 @@
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
+      <c r="AL8" t="n">
+        <v>462.21</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>25.6</v>
+      </c>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
@@ -2276,7 +2280,9 @@
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
+      <c r="AL9" t="n">
+        <v>444.58</v>
+      </c>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
@@ -2447,8 +2453,12 @@
       </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AL10" t="n">
+        <v>461.81</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>65.73</v>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
@@ -2638,8 +2648,12 @@
       </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
+      <c r="AL11" t="n">
+        <v>452.38</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>16.12</v>
+      </c>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
@@ -2833,8 +2847,12 @@
       </c>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
+      <c r="AL12" t="n">
+        <v>276.6</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>45.98</v>
+      </c>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
@@ -3024,8 +3042,12 @@
       </c>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
+      <c r="AL13" t="n">
+        <v>303.57</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>21.05</v>
+      </c>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
@@ -3215,8 +3237,12 @@
       </c>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
+      <c r="AL14" t="n">
+        <v>263.47</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>4.56</v>
+      </c>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
@@ -3406,8 +3432,12 @@
       </c>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
+      <c r="AL15" t="n">
+        <v>248.34</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>11.95</v>
+      </c>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
@@ -4497,8 +4527,12 @@
       </c>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
-      <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="inlineStr"/>
+      <c r="AL20" t="n">
+        <v>517.2</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>36.65</v>
+      </c>
       <c r="AN20" t="inlineStr"/>
       <c r="AO20" t="inlineStr"/>
       <c r="AP20" t="inlineStr"/>
@@ -4688,8 +4722,12 @@
       </c>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
-      <c r="AL21" t="inlineStr"/>
-      <c r="AM21" t="inlineStr"/>
+      <c r="AL21" t="n">
+        <v>567.65</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>103.37</v>
+      </c>
       <c r="AN21" t="inlineStr"/>
       <c r="AO21" t="inlineStr"/>
       <c r="AP21" t="inlineStr"/>
@@ -4879,8 +4917,12 @@
       </c>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
-      <c r="AM22" t="inlineStr"/>
+      <c r="AL22" t="n">
+        <v>498.3</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>49.19</v>
+      </c>
       <c r="AN22" t="inlineStr"/>
       <c r="AO22" t="inlineStr"/>
       <c r="AP22" t="inlineStr"/>
@@ -5070,8 +5112,12 @@
       </c>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
-      <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
+      <c r="AL23" t="n">
+        <v>497.57</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>47.07</v>
+      </c>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
@@ -5265,8 +5311,12 @@
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
+      <c r="AL24" t="n">
+        <v>458.37</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>24.12</v>
+      </c>
       <c r="AN24" t="inlineStr"/>
       <c r="AO24" t="inlineStr"/>
       <c r="AP24" t="inlineStr"/>
@@ -5456,8 +5506,12 @@
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
-      <c r="AM25" t="inlineStr"/>
+      <c r="AL25" t="n">
+        <v>484.91</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>63.86</v>
+      </c>
       <c r="AN25" t="inlineStr"/>
       <c r="AO25" t="inlineStr"/>
       <c r="AP25" t="inlineStr"/>
@@ -5647,8 +5701,12 @@
       </c>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
-      <c r="AL26" t="inlineStr"/>
-      <c r="AM26" t="inlineStr"/>
+      <c r="AL26" t="n">
+        <v>447.24</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>11.29</v>
+      </c>
       <c r="AN26" t="inlineStr"/>
       <c r="AO26" t="inlineStr"/>
       <c r="AP26" t="inlineStr"/>
@@ -5838,8 +5896,12 @@
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-      <c r="AL27" t="inlineStr"/>
-      <c r="AM27" t="inlineStr"/>
+      <c r="AL27" t="n">
+        <v>450.2</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>29.2</v>
+      </c>
       <c r="AN27" t="inlineStr"/>
       <c r="AO27" t="inlineStr"/>
       <c r="AP27" t="inlineStr"/>

</xml_diff>

<commit_message>
editado preliminar y falta el grafico per elevation
</commit_message>
<xml_diff>
--- a/Summary.xlsx
+++ b/Summary.xlsx
@@ -566,139 +566,139 @@
       <c r="AE1" s="1" t="n"/>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Specific leaf area (g/cm²)</t>
+          <t>area_basal_m2</t>
         </is>
       </c>
       <c r="AG1" s="1" t="n"/>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>area_basal_m2</t>
+          <t>sample-ID</t>
         </is>
       </c>
       <c r="AI1" s="1" t="n"/>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>sample-ID</t>
+          <t>number of leaves</t>
         </is>
       </c>
       <c r="AK1" s="1" t="n"/>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>number of leaves</t>
+          <t>dry matter content (mg/g)</t>
         </is>
       </c>
       <c r="AM1" s="1" t="n"/>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>dry matter content (mg/g)</t>
+          <t>C (mg/g)</t>
         </is>
       </c>
       <c r="AO1" s="1" t="n"/>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>C (mg/g)</t>
+          <t>N (mg/g)</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="n"/>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>N (mg/g)</t>
+          <t>P (mg/g)</t>
         </is>
       </c>
       <c r="AS1" s="1" t="n"/>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>P (mg/g)</t>
+          <t>Al (mg/g)</t>
         </is>
       </c>
       <c r="AU1" s="1" t="n"/>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>Al (mg/g)</t>
+          <t>Ca (mg/g)</t>
         </is>
       </c>
       <c r="AW1" s="1" t="n"/>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>Ca (mg/g)</t>
+          <t>Fe (mg/g)</t>
         </is>
       </c>
       <c r="AY1" s="1" t="n"/>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>Fe (mg/g)</t>
+          <t>K (mg/g)</t>
         </is>
       </c>
       <c r="BA1" s="1" t="n"/>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>K (mg/g)</t>
+          <t>Mg (mg/g)</t>
         </is>
       </c>
       <c r="BC1" s="1" t="n"/>
       <c r="BD1" s="1" t="inlineStr">
         <is>
-          <t>Mg (mg/g)</t>
+          <t>Na (mg/g)</t>
         </is>
       </c>
       <c r="BE1" s="1" t="n"/>
       <c r="BF1" s="1" t="inlineStr">
         <is>
-          <t>Na (mg/g)</t>
+          <t>S (mg/g)</t>
         </is>
       </c>
       <c r="BG1" s="1" t="n"/>
       <c r="BH1" s="1" t="inlineStr">
         <is>
-          <t>S (mg/g)</t>
+          <t>△13C_cell</t>
         </is>
       </c>
       <c r="BI1" s="1" t="n"/>
       <c r="BJ1" s="1" t="inlineStr">
         <is>
-          <t>△13C_cell</t>
+          <t>Ci</t>
         </is>
       </c>
       <c r="BK1" s="1" t="n"/>
       <c r="BL1" s="1" t="inlineStr">
         <is>
-          <t>Ci</t>
+          <t>Ci/Ca</t>
         </is>
       </c>
       <c r="BM1" s="1" t="n"/>
       <c r="BN1" s="1" t="inlineStr">
         <is>
-          <t>Ci/Ca</t>
+          <t>iWUE (μmol/mol)</t>
         </is>
       </c>
       <c r="BO1" s="1" t="n"/>
       <c r="BP1" s="1" t="inlineStr">
         <is>
-          <t>iWUE (μmol/mol)</t>
+          <t>annual_precipitation_mm</t>
         </is>
       </c>
       <c r="BQ1" s="1" t="n"/>
       <c r="BR1" s="1" t="inlineStr">
         <is>
-          <t>annual_precipitation_mm</t>
+          <t>elevation_m</t>
         </is>
       </c>
       <c r="BS1" s="1" t="n"/>
       <c r="BT1" s="1" t="inlineStr">
         <is>
-          <t>elevation_m</t>
+          <t>mean_annual_temperature_C</t>
         </is>
       </c>
       <c r="BU1" s="1" t="n"/>
       <c r="BV1" s="1" t="inlineStr">
         <is>
-          <t>mean_annual_temperature_C</t>
+          <t>WD</t>
         </is>
       </c>
       <c r="BW1" s="1" t="n"/>
       <c r="BX1" s="1" t="inlineStr">
         <is>
-          <t>WD</t>
+          <t>Specific leaf area (g/cm²)</t>
         </is>
       </c>
       <c r="BY1" s="1" t="n"/>
@@ -1267,115 +1267,115 @@
       <c r="AE4" t="n">
         <v>148.92</v>
       </c>
-      <c r="AF4" t="n">
-        <v>35.39</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>4.16</v>
-      </c>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="n">
+        <v>592166.17</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>131.93</v>
+      </c>
       <c r="AJ4" t="n">
-        <v>592166.17</v>
+        <v>20</v>
       </c>
       <c r="AK4" t="n">
-        <v>131.93</v>
+        <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>20</v>
+        <v>458.84</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>40.17</v>
       </c>
       <c r="AN4" t="n">
-        <v>458.84</v>
+        <v>510.89</v>
       </c>
       <c r="AO4" t="n">
-        <v>40.17</v>
+        <v>13.98</v>
       </c>
       <c r="AP4" t="n">
-        <v>510.89</v>
+        <v>12.75</v>
       </c>
       <c r="AQ4" t="n">
-        <v>13.98</v>
+        <v>2.04</v>
       </c>
       <c r="AR4" t="n">
-        <v>12.75</v>
+        <v>0.89</v>
       </c>
       <c r="AS4" t="n">
-        <v>2.04</v>
+        <v>0.43</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.89</v>
+        <v>0.04</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.43</v>
+        <v>0.04</v>
       </c>
       <c r="AV4" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>17.56</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>288.48</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="BM4" t="n">
         <v>0.04</v>
       </c>
-      <c r="AW4" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="BG4" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>17.56</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>288.48</v>
-      </c>
-      <c r="BM4" t="n">
-        <v>18.81</v>
-      </c>
       <c r="BN4" t="n">
-        <v>0.63</v>
+        <v>106.54</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.04</v>
+        <v>11.75</v>
       </c>
       <c r="BP4" t="n">
-        <v>106.54</v>
+        <v>2000</v>
       </c>
       <c r="BQ4" t="n">
-        <v>11.75</v>
+        <v>0</v>
       </c>
       <c r="BR4" t="n">
         <v>2000</v>
@@ -1384,22 +1384,22 @@
         <v>0</v>
       </c>
       <c r="BT4" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU4" t="n">
         <v>0</v>
       </c>
       <c r="BV4" t="n">
-        <v>15</v>
+        <v>0.52</v>
       </c>
       <c r="BW4" t="n">
         <v>0</v>
       </c>
       <c r="BX4" t="n">
-        <v>0.52</v>
+        <v>35.39</v>
       </c>
       <c r="BY4" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="BZ4" t="n">
         <v>0.54</v>
@@ -1522,115 +1522,115 @@
       <c r="AE5" t="n">
         <v>208.63</v>
       </c>
-      <c r="AF5" t="n">
-        <v>35.34</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>4.79</v>
-      </c>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="n">
+        <v>592154.89</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>91.08</v>
+      </c>
       <c r="AJ5" t="n">
-        <v>592154.89</v>
+        <v>20</v>
       </c>
       <c r="AK5" t="n">
-        <v>91.08</v>
+        <v>0</v>
       </c>
       <c r="AL5" t="n">
-        <v>20</v>
+        <v>436.5</v>
       </c>
       <c r="AM5" t="n">
-        <v>0</v>
+        <v>43.22</v>
       </c>
       <c r="AN5" t="n">
-        <v>436.5</v>
+        <v>512.6900000000001</v>
       </c>
       <c r="AO5" t="n">
-        <v>43.22</v>
+        <v>9.93</v>
       </c>
       <c r="AP5" t="n">
-        <v>512.6900000000001</v>
+        <v>11.67</v>
       </c>
       <c r="AQ5" t="n">
-        <v>9.93</v>
+        <v>1.6</v>
       </c>
       <c r="AR5" t="n">
-        <v>11.67</v>
+        <v>1.26</v>
       </c>
       <c r="AS5" t="n">
-        <v>1.6</v>
+        <v>0.26</v>
       </c>
       <c r="AT5" t="n">
-        <v>1.26</v>
+        <v>0.01</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.26</v>
+        <v>0.01</v>
       </c>
       <c r="AV5" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AY5" t="n">
         <v>0.01</v>
       </c>
-      <c r="AW5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AX5" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="AY5" t="n">
-        <v>1.4</v>
-      </c>
       <c r="AZ5" t="n">
-        <v>0.02</v>
+        <v>4.49</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.01</v>
+        <v>1.41</v>
       </c>
       <c r="BB5" t="n">
-        <v>4.49</v>
+        <v>2.11</v>
       </c>
       <c r="BC5" t="n">
-        <v>1.41</v>
+        <v>0.57</v>
       </c>
       <c r="BD5" t="n">
-        <v>2.11</v>
+        <v>0.03</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.57</v>
+        <v>0.05</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.03</v>
+        <v>0.62</v>
       </c>
       <c r="BG5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>293.36</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>22.36</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="BM5" t="n">
         <v>0.05</v>
       </c>
-      <c r="BH5" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="BI5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="BJ5" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>293.36</v>
-      </c>
-      <c r="BM5" t="n">
-        <v>22.36</v>
-      </c>
       <c r="BN5" t="n">
-        <v>0.64</v>
+        <v>103.5</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.05</v>
+        <v>13.97</v>
       </c>
       <c r="BP5" t="n">
-        <v>103.5</v>
+        <v>2000</v>
       </c>
       <c r="BQ5" t="n">
-        <v>13.97</v>
+        <v>0</v>
       </c>
       <c r="BR5" t="n">
         <v>2000</v>
@@ -1639,22 +1639,22 @@
         <v>0</v>
       </c>
       <c r="BT5" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU5" t="n">
         <v>0</v>
       </c>
       <c r="BV5" t="n">
-        <v>15</v>
+        <v>0.52</v>
       </c>
       <c r="BW5" t="n">
         <v>0</v>
       </c>
       <c r="BX5" t="n">
-        <v>0.52</v>
+        <v>35.34</v>
       </c>
       <c r="BY5" t="n">
-        <v>0</v>
+        <v>4.79</v>
       </c>
       <c r="BZ5" t="n">
         <v>0.5600000000000001</v>
@@ -1777,115 +1777,115 @@
       <c r="AE6" t="n">
         <v>151.86</v>
       </c>
-      <c r="AF6" t="n">
-        <v>36.46</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="n">
+        <v>592184.38</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>102.74</v>
+      </c>
       <c r="AJ6" t="n">
-        <v>592184.38</v>
+        <v>20</v>
       </c>
       <c r="AK6" t="n">
-        <v>102.74</v>
+        <v>0</v>
       </c>
       <c r="AL6" t="n">
-        <v>20</v>
+        <v>443.24</v>
       </c>
       <c r="AM6" t="n">
-        <v>0</v>
+        <v>46.75</v>
       </c>
       <c r="AN6" t="n">
-        <v>443.24</v>
+        <v>509.58</v>
       </c>
       <c r="AO6" t="n">
-        <v>46.75</v>
+        <v>15.91</v>
       </c>
       <c r="AP6" t="n">
-        <v>509.58</v>
+        <v>13.03</v>
       </c>
       <c r="AQ6" t="n">
-        <v>15.91</v>
+        <v>2.6</v>
       </c>
       <c r="AR6" t="n">
-        <v>13.03</v>
+        <v>0.83</v>
       </c>
       <c r="AS6" t="n">
-        <v>2.6</v>
+        <v>0.45</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.83</v>
+        <v>0.02</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.45</v>
+        <v>0.02</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.02</v>
+        <v>2.42</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.02</v>
+        <v>1.58</v>
       </c>
       <c r="AX6" t="n">
-        <v>2.42</v>
+        <v>0.05</v>
       </c>
       <c r="AY6" t="n">
-        <v>1.58</v>
+        <v>0.05</v>
       </c>
       <c r="AZ6" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BE6" t="n">
         <v>0.05</v>
       </c>
-      <c r="BA6" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>3.64</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>1.21</v>
-      </c>
       <c r="BF6" t="n">
-        <v>0.03</v>
+        <v>0.67</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.67</v>
+        <v>17.83</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.4</v>
+        <v>1.52</v>
       </c>
       <c r="BJ6" t="n">
-        <v>17.83</v>
+        <v>293.97</v>
       </c>
       <c r="BK6" t="n">
-        <v>1.52</v>
+        <v>30.77</v>
       </c>
       <c r="BL6" t="n">
-        <v>293.97</v>
+        <v>0.64</v>
       </c>
       <c r="BM6" t="n">
-        <v>30.77</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.64</v>
+        <v>103.12</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.07000000000000001</v>
+        <v>19.23</v>
       </c>
       <c r="BP6" t="n">
-        <v>103.12</v>
+        <v>2000</v>
       </c>
       <c r="BQ6" t="n">
-        <v>19.23</v>
+        <v>0</v>
       </c>
       <c r="BR6" t="n">
         <v>2000</v>
@@ -1894,22 +1894,22 @@
         <v>0</v>
       </c>
       <c r="BT6" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU6" t="n">
         <v>0</v>
       </c>
       <c r="BV6" t="n">
-        <v>15</v>
+        <v>0.52</v>
       </c>
       <c r="BW6" t="n">
         <v>0</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.52</v>
+        <v>36.46</v>
       </c>
       <c r="BY6" t="n">
-        <v>0</v>
+        <v>3.96</v>
       </c>
       <c r="BZ6" t="n">
         <v>0.5600000000000001</v>
@@ -2032,115 +2032,115 @@
       <c r="AE7" t="n">
         <v>157.74</v>
       </c>
-      <c r="AF7" t="n">
-        <v>35.91</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="n">
+        <v>592154.27</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>103.52</v>
+      </c>
       <c r="AJ7" t="n">
-        <v>592154.27</v>
+        <v>20</v>
       </c>
       <c r="AK7" t="n">
-        <v>103.52</v>
+        <v>0</v>
       </c>
       <c r="AL7" t="n">
-        <v>20</v>
+        <v>445.05</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>31.92</v>
       </c>
       <c r="AN7" t="n">
-        <v>445.05</v>
+        <v>506.63</v>
       </c>
       <c r="AO7" t="n">
-        <v>31.92</v>
+        <v>11.49</v>
       </c>
       <c r="AP7" t="n">
-        <v>506.63</v>
+        <v>13.43</v>
       </c>
       <c r="AQ7" t="n">
-        <v>11.49</v>
+        <v>2.12</v>
       </c>
       <c r="AR7" t="n">
-        <v>13.43</v>
+        <v>1.2</v>
       </c>
       <c r="AS7" t="n">
-        <v>2.12</v>
+        <v>0.82</v>
       </c>
       <c r="AT7" t="n">
-        <v>1.2</v>
+        <v>0.03</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.82</v>
+        <v>0.04</v>
       </c>
       <c r="AV7" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="AX7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AW7" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>3.62</v>
-      </c>
       <c r="AY7" t="n">
-        <v>2.14</v>
+        <v>0.02</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.03</v>
+        <v>4.38</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.02</v>
+        <v>1.38</v>
       </c>
       <c r="BB7" t="n">
-        <v>4.38</v>
+        <v>2.02</v>
       </c>
       <c r="BC7" t="n">
-        <v>1.38</v>
+        <v>0.67</v>
       </c>
       <c r="BD7" t="n">
-        <v>2.02</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.67</v>
+        <v>0.09</v>
       </c>
       <c r="BF7" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>18.13</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>300.04</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="BM7" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="BG7" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="BJ7" t="n">
-        <v>18.13</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>300.04</v>
-      </c>
-      <c r="BM7" t="n">
-        <v>32.01</v>
-      </c>
       <c r="BN7" t="n">
-        <v>0.65</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.07000000000000001</v>
+        <v>20.01</v>
       </c>
       <c r="BP7" t="n">
-        <v>99.31999999999999</v>
+        <v>2000</v>
       </c>
       <c r="BQ7" t="n">
-        <v>20.01</v>
+        <v>0</v>
       </c>
       <c r="BR7" t="n">
         <v>2000</v>
@@ -2149,22 +2149,22 @@
         <v>0</v>
       </c>
       <c r="BT7" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU7" t="n">
         <v>0</v>
       </c>
       <c r="BV7" t="n">
-        <v>15</v>
+        <v>0.52</v>
       </c>
       <c r="BW7" t="n">
         <v>0</v>
       </c>
       <c r="BX7" t="n">
-        <v>0.52</v>
+        <v>35.91</v>
       </c>
       <c r="BY7" t="n">
-        <v>0</v>
+        <v>3.67</v>
       </c>
       <c r="BZ7" t="n">
         <v>0.55</v>
@@ -2296,27 +2296,23 @@
         <v>252.02</v>
       </c>
       <c r="AF8" t="n">
-        <v>92.05</v>
+        <v>0.05</v>
       </c>
       <c r="AG8" t="n">
-        <v>10.83</v>
-      </c>
-      <c r="AH8" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI8" t="n">
-        <v>0.05</v>
-      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="n">
+      <c r="AL8" t="n">
         <v>462.21</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="AM8" t="n">
         <v>25.6</v>
       </c>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
@@ -2335,55 +2331,59 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
+      <c r="BH8" t="n">
+        <v>21.88</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0.45</v>
+      </c>
       <c r="BJ8" t="n">
-        <v>21.88</v>
+        <v>376.21</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.45</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BL8" t="n">
-        <v>376.21</v>
+        <v>0.82</v>
       </c>
       <c r="BM8" t="n">
-        <v>9.039999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.82</v>
+        <v>51.71</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.02</v>
+        <v>5.65</v>
       </c>
       <c r="BP8" t="n">
-        <v>51.71</v>
+        <v>2000</v>
       </c>
       <c r="BQ8" t="n">
-        <v>5.65</v>
+        <v>0</v>
       </c>
       <c r="BR8" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS8" t="n">
         <v>0</v>
       </c>
       <c r="BT8" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU8" t="n">
         <v>0</v>
       </c>
       <c r="BV8" t="n">
-        <v>19</v>
+        <v>0.58</v>
       </c>
       <c r="BW8" t="n">
         <v>0</v>
       </c>
       <c r="BX8" t="n">
-        <v>0.58</v>
+        <v>92.05</v>
       </c>
       <c r="BY8" t="n">
-        <v>0</v>
+        <v>10.83</v>
       </c>
       <c r="BZ8" t="n">
         <v>0.54</v>
@@ -2483,20 +2483,18 @@
       </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="n">
-        <v>112.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+      <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
+      <c r="AL9" t="n">
+        <v>444.58</v>
+      </c>
       <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="n">
-        <v>444.58</v>
-      </c>
+      <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr"/>
@@ -2516,38 +2514,40 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="inlineStr"/>
-      <c r="BH9" t="inlineStr"/>
+      <c r="BH9" t="n">
+        <v>23.11</v>
+      </c>
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="n">
-        <v>23.11</v>
+        <v>401.28</v>
       </c>
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="n">
-        <v>401.28</v>
+        <v>0.87</v>
       </c>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>0.87</v>
+        <v>36.04</v>
       </c>
       <c r="BO9" t="inlineStr"/>
       <c r="BP9" t="n">
-        <v>36.04</v>
+        <v>2000</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="n">
-        <v>19</v>
+        <v>0.58</v>
       </c>
       <c r="BW9" t="inlineStr"/>
       <c r="BX9" t="n">
-        <v>0.58</v>
+        <v>112.06</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="n">
@@ -2666,27 +2666,23 @@
         <v>95.02</v>
       </c>
       <c r="AF10" t="n">
-        <v>91.5</v>
+        <v>0.05</v>
       </c>
       <c r="AG10" t="n">
-        <v>38.65</v>
-      </c>
-      <c r="AH10" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AI10" t="n">
         <v>0.03</v>
       </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="n">
+      <c r="AL10" t="n">
         <v>461.81</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="AM10" t="n">
         <v>65.73</v>
       </c>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
@@ -2705,55 +2701,59 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="inlineStr"/>
-      <c r="BH10" t="inlineStr"/>
-      <c r="BI10" t="inlineStr"/>
+      <c r="BH10" t="n">
+        <v>22.14</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>0.38</v>
+      </c>
       <c r="BJ10" t="n">
-        <v>22.14</v>
+        <v>381.45</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.38</v>
+        <v>7.72</v>
       </c>
       <c r="BL10" t="n">
-        <v>381.45</v>
+        <v>0.83</v>
       </c>
       <c r="BM10" t="n">
-        <v>7.72</v>
+        <v>0.02</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.83</v>
+        <v>48.44</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.02</v>
+        <v>4.83</v>
       </c>
       <c r="BP10" t="n">
-        <v>48.44</v>
+        <v>2000</v>
       </c>
       <c r="BQ10" t="n">
-        <v>4.83</v>
+        <v>0</v>
       </c>
       <c r="BR10" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS10" t="n">
         <v>0</v>
       </c>
       <c r="BT10" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU10" t="n">
         <v>0</v>
       </c>
       <c r="BV10" t="n">
-        <v>19</v>
+        <v>0.58</v>
       </c>
       <c r="BW10" t="n">
         <v>0</v>
       </c>
       <c r="BX10" t="n">
-        <v>0.58</v>
+        <v>91.5</v>
       </c>
       <c r="BY10" t="n">
-        <v>0</v>
+        <v>38.65</v>
       </c>
       <c r="BZ10" t="n">
         <v>0.54</v>
@@ -2881,27 +2881,23 @@
         <v>70.29000000000001</v>
       </c>
       <c r="AF11" t="n">
-        <v>95.65000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="AG11" t="n">
-        <v>6.27</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AI11" t="n">
         <v>0.04</v>
       </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
-      <c r="AN11" t="n">
+      <c r="AL11" t="n">
         <v>452.38</v>
       </c>
-      <c r="AO11" t="n">
+      <c r="AM11" t="n">
         <v>16.12</v>
       </c>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="inlineStr"/>
@@ -2920,55 +2916,59 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="inlineStr"/>
-      <c r="BH11" t="inlineStr"/>
-      <c r="BI11" t="inlineStr"/>
+      <c r="BH11" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>1.3</v>
+      </c>
       <c r="BJ11" t="n">
-        <v>21.05</v>
+        <v>359.39</v>
       </c>
       <c r="BK11" t="n">
-        <v>1.3</v>
+        <v>26.48</v>
       </c>
       <c r="BL11" t="n">
-        <v>359.39</v>
+        <v>0.78</v>
       </c>
       <c r="BM11" t="n">
-        <v>26.48</v>
+        <v>0.06</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.78</v>
+        <v>62.23</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.06</v>
+        <v>16.55</v>
       </c>
       <c r="BP11" t="n">
-        <v>62.23</v>
+        <v>2000</v>
       </c>
       <c r="BQ11" t="n">
-        <v>16.55</v>
+        <v>0</v>
       </c>
       <c r="BR11" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS11" t="n">
         <v>0</v>
       </c>
       <c r="BT11" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU11" t="n">
         <v>0</v>
       </c>
       <c r="BV11" t="n">
-        <v>19</v>
+        <v>0.58</v>
       </c>
       <c r="BW11" t="n">
         <v>0</v>
       </c>
       <c r="BX11" t="n">
-        <v>0.58</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="BY11" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="BZ11" t="n">
         <v>0.55</v>
@@ -3100,27 +3100,23 @@
         <v>26.75</v>
       </c>
       <c r="AF12" t="n">
-        <v>68.88</v>
+        <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>16.18</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="n">
+      <c r="AL12" t="n">
         <v>276.6</v>
       </c>
-      <c r="AO12" t="n">
+      <c r="AM12" t="n">
         <v>45.98</v>
       </c>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
@@ -3139,55 +3135,59 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="inlineStr"/>
-      <c r="BH12" t="inlineStr"/>
-      <c r="BI12" t="inlineStr"/>
+      <c r="BH12" t="n">
+        <v>17.87</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>1.51</v>
+      </c>
       <c r="BJ12" t="n">
-        <v>17.87</v>
+        <v>294.7</v>
       </c>
       <c r="BK12" t="n">
-        <v>1.51</v>
+        <v>30.67</v>
       </c>
       <c r="BL12" t="n">
-        <v>294.7</v>
+        <v>0.64</v>
       </c>
       <c r="BM12" t="n">
-        <v>30.67</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.64</v>
+        <v>102.66</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.07000000000000001</v>
+        <v>19.17</v>
       </c>
       <c r="BP12" t="n">
-        <v>102.66</v>
+        <v>4500</v>
       </c>
       <c r="BQ12" t="n">
-        <v>19.17</v>
+        <v>0</v>
       </c>
       <c r="BR12" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS12" t="n">
         <v>0</v>
       </c>
       <c r="BT12" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU12" t="n">
         <v>0</v>
       </c>
       <c r="BV12" t="n">
-        <v>10</v>
+        <v>0.58</v>
       </c>
       <c r="BW12" t="n">
         <v>0</v>
       </c>
       <c r="BX12" t="n">
-        <v>0.58</v>
+        <v>68.88</v>
       </c>
       <c r="BY12" t="n">
-        <v>0</v>
+        <v>16.18</v>
       </c>
       <c r="BZ12" t="n">
         <v>0.72</v>
@@ -3315,27 +3315,23 @@
         <v>117.09</v>
       </c>
       <c r="AF13" t="n">
-        <v>60.87</v>
+        <v>0.02</v>
       </c>
       <c r="AG13" t="n">
-        <v>6.61</v>
-      </c>
-      <c r="AH13" t="n">
         <v>0.02</v>
       </c>
-      <c r="AI13" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
-      <c r="AN13" t="n">
+      <c r="AL13" t="n">
         <v>303.57</v>
       </c>
-      <c r="AO13" t="n">
+      <c r="AM13" t="n">
         <v>21.05</v>
       </c>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
@@ -3354,55 +3350,59 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="inlineStr"/>
-      <c r="BH13" t="inlineStr"/>
-      <c r="BI13" t="inlineStr"/>
+      <c r="BH13" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>2.15</v>
+      </c>
       <c r="BJ13" t="n">
-        <v>17.39</v>
+        <v>285.13</v>
       </c>
       <c r="BK13" t="n">
-        <v>2.15</v>
+        <v>43.7</v>
       </c>
       <c r="BL13" t="n">
-        <v>285.13</v>
+        <v>0.62</v>
       </c>
       <c r="BM13" t="n">
-        <v>43.7</v>
+        <v>0.1</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.62</v>
+        <v>108.64</v>
       </c>
       <c r="BO13" t="n">
-        <v>0.1</v>
+        <v>27.31</v>
       </c>
       <c r="BP13" t="n">
-        <v>108.64</v>
+        <v>4500</v>
       </c>
       <c r="BQ13" t="n">
-        <v>27.31</v>
+        <v>0</v>
       </c>
       <c r="BR13" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS13" t="n">
         <v>0</v>
       </c>
       <c r="BT13" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU13" t="n">
         <v>0</v>
       </c>
       <c r="BV13" t="n">
-        <v>10</v>
+        <v>0.58</v>
       </c>
       <c r="BW13" t="n">
         <v>0</v>
       </c>
       <c r="BX13" t="n">
-        <v>0.58</v>
+        <v>60.87</v>
       </c>
       <c r="BY13" t="n">
-        <v>0</v>
+        <v>6.61</v>
       </c>
       <c r="BZ13" t="n">
         <v>0.7</v>
@@ -3530,27 +3530,23 @@
         <v>55.44</v>
       </c>
       <c r="AF14" t="n">
-        <v>65.98</v>
+        <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
-      <c r="AN14" t="n">
+      <c r="AL14" t="n">
         <v>263.47</v>
       </c>
-      <c r="AO14" t="n">
+      <c r="AM14" t="n">
         <v>4.56</v>
       </c>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
@@ -3569,55 +3565,59 @@
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="inlineStr"/>
-      <c r="BH14" t="inlineStr"/>
-      <c r="BI14" t="inlineStr"/>
+      <c r="BH14" t="n">
+        <v>15.82</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>1.32</v>
+      </c>
       <c r="BJ14" t="n">
-        <v>15.82</v>
+        <v>253.23</v>
       </c>
       <c r="BK14" t="n">
-        <v>1.32</v>
+        <v>26.77</v>
       </c>
       <c r="BL14" t="n">
-        <v>253.23</v>
+        <v>0.55</v>
       </c>
       <c r="BM14" t="n">
-        <v>26.77</v>
+        <v>0.06</v>
       </c>
       <c r="BN14" t="n">
-        <v>0.55</v>
+        <v>128.58</v>
       </c>
       <c r="BO14" t="n">
-        <v>0.06</v>
+        <v>16.73</v>
       </c>
       <c r="BP14" t="n">
-        <v>128.58</v>
+        <v>4500</v>
       </c>
       <c r="BQ14" t="n">
-        <v>16.73</v>
+        <v>0</v>
       </c>
       <c r="BR14" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS14" t="n">
         <v>0</v>
       </c>
       <c r="BT14" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU14" t="n">
         <v>0</v>
       </c>
       <c r="BV14" t="n">
-        <v>10</v>
+        <v>0.58</v>
       </c>
       <c r="BW14" t="n">
         <v>0</v>
       </c>
       <c r="BX14" t="n">
-        <v>0.58</v>
+        <v>65.98</v>
       </c>
       <c r="BY14" t="n">
-        <v>0</v>
+        <v>5.04</v>
       </c>
       <c r="BZ14" t="n">
         <v>0.74</v>
@@ -3745,27 +3745,23 @@
         <v>97.78</v>
       </c>
       <c r="AF15" t="n">
-        <v>75.91</v>
+        <v>0</v>
       </c>
       <c r="AG15" t="n">
-        <v>12.42</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
-      <c r="AN15" t="n">
+      <c r="AL15" t="n">
         <v>248.34</v>
       </c>
-      <c r="AO15" t="n">
+      <c r="AM15" t="n">
         <v>11.95</v>
       </c>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
       <c r="AQ15" t="inlineStr"/>
       <c r="AR15" t="inlineStr"/>
@@ -3784,55 +3780,59 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="inlineStr"/>
-      <c r="BH15" t="inlineStr"/>
-      <c r="BI15" t="inlineStr"/>
+      <c r="BH15" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>1.66</v>
+      </c>
       <c r="BJ15" t="n">
-        <v>18.37</v>
+        <v>304.97</v>
       </c>
       <c r="BK15" t="n">
-        <v>1.66</v>
+        <v>33.73</v>
       </c>
       <c r="BL15" t="n">
-        <v>304.97</v>
+        <v>0.66</v>
       </c>
       <c r="BM15" t="n">
-        <v>33.73</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="BN15" t="n">
-        <v>0.66</v>
+        <v>96.23999999999999</v>
       </c>
       <c r="BO15" t="n">
-        <v>0.07000000000000001</v>
+        <v>21.08</v>
       </c>
       <c r="BP15" t="n">
-        <v>96.23999999999999</v>
+        <v>4500</v>
       </c>
       <c r="BQ15" t="n">
-        <v>21.08</v>
+        <v>0</v>
       </c>
       <c r="BR15" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS15" t="n">
         <v>0</v>
       </c>
       <c r="BT15" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU15" t="n">
         <v>0</v>
       </c>
       <c r="BV15" t="n">
-        <v>10</v>
+        <v>0.58</v>
       </c>
       <c r="BW15" t="n">
         <v>0</v>
       </c>
       <c r="BX15" t="n">
-        <v>0.58</v>
+        <v>75.91</v>
       </c>
       <c r="BY15" t="n">
-        <v>0</v>
+        <v>12.42</v>
       </c>
       <c r="BZ15" t="n">
         <v>0.75</v>
@@ -3959,115 +3959,115 @@
       <c r="AE16" t="n">
         <v>138.78</v>
       </c>
-      <c r="AF16" t="n">
-        <v>37.13</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="n">
+        <v>592162.27</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>130.48</v>
+      </c>
       <c r="AJ16" t="n">
-        <v>592162.27</v>
+        <v>20</v>
       </c>
       <c r="AK16" t="n">
-        <v>130.48</v>
+        <v>0</v>
       </c>
       <c r="AL16" t="n">
-        <v>20</v>
+        <v>479.82</v>
       </c>
       <c r="AM16" t="n">
-        <v>0</v>
+        <v>36.04</v>
       </c>
       <c r="AN16" t="n">
-        <v>479.82</v>
+        <v>497.47</v>
       </c>
       <c r="AO16" t="n">
-        <v>36.04</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="AP16" t="n">
-        <v>497.47</v>
+        <v>12.69</v>
       </c>
       <c r="AQ16" t="n">
-        <v>8.279999999999999</v>
+        <v>4.66</v>
       </c>
       <c r="AR16" t="n">
-        <v>12.69</v>
+        <v>0.52</v>
       </c>
       <c r="AS16" t="n">
-        <v>4.66</v>
+        <v>0.22</v>
       </c>
       <c r="AT16" t="n">
-        <v>0.52</v>
+        <v>0.41</v>
       </c>
       <c r="AU16" t="n">
-        <v>0.22</v>
+        <v>1.37</v>
       </c>
       <c r="AV16" t="n">
-        <v>0.41</v>
+        <v>1.39</v>
       </c>
       <c r="AW16" t="n">
-        <v>1.37</v>
+        <v>1.17</v>
       </c>
       <c r="AX16" t="n">
-        <v>1.39</v>
+        <v>0.06</v>
       </c>
       <c r="AY16" t="n">
-        <v>1.17</v>
+        <v>0.02</v>
       </c>
       <c r="AZ16" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BE16" t="n">
         <v>0.06</v>
       </c>
-      <c r="BA16" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="BB16" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="BC16" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="BD16" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="BE16" t="n">
-        <v>0.64</v>
-      </c>
       <c r="BF16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>315.7</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="BM16" t="n">
         <v>0.05</v>
       </c>
-      <c r="BG16" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="BH16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="BI16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="BJ16" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="BK16" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="BL16" t="n">
-        <v>315.7</v>
-      </c>
-      <c r="BM16" t="n">
-        <v>24.52</v>
-      </c>
       <c r="BN16" t="n">
-        <v>0.6899999999999999</v>
+        <v>89.53</v>
       </c>
       <c r="BO16" t="n">
-        <v>0.05</v>
+        <v>15.32</v>
       </c>
       <c r="BP16" t="n">
-        <v>89.53</v>
+        <v>2000</v>
       </c>
       <c r="BQ16" t="n">
-        <v>15.32</v>
+        <v>0</v>
       </c>
       <c r="BR16" t="n">
         <v>2000</v>
@@ -4076,22 +4076,22 @@
         <v>0</v>
       </c>
       <c r="BT16" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU16" t="n">
         <v>0</v>
       </c>
       <c r="BV16" t="n">
-        <v>15</v>
+        <v>0.72</v>
       </c>
       <c r="BW16" t="n">
         <v>0</v>
       </c>
       <c r="BX16" t="n">
-        <v>0.72</v>
+        <v>37.13</v>
       </c>
       <c r="BY16" t="n">
-        <v>0</v>
+        <v>3.92</v>
       </c>
       <c r="BZ16" t="n">
         <v>0.52</v>
@@ -4214,115 +4214,115 @@
       <c r="AE17" t="n">
         <v>141.02</v>
       </c>
-      <c r="AF17" t="n">
-        <v>34.39</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="n">
+        <v>592190.7</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>124.79</v>
+      </c>
       <c r="AJ17" t="n">
-        <v>592190.7</v>
+        <v>20</v>
       </c>
       <c r="AK17" t="n">
-        <v>124.79</v>
+        <v>0</v>
       </c>
       <c r="AL17" t="n">
-        <v>20</v>
+        <v>465.81</v>
       </c>
       <c r="AM17" t="n">
-        <v>0</v>
+        <v>30.98</v>
       </c>
       <c r="AN17" t="n">
-        <v>465.81</v>
+        <v>499.64</v>
       </c>
       <c r="AO17" t="n">
-        <v>30.98</v>
+        <v>11.64</v>
       </c>
       <c r="AP17" t="n">
-        <v>499.64</v>
+        <v>11.29</v>
       </c>
       <c r="AQ17" t="n">
-        <v>11.64</v>
+        <v>0.89</v>
       </c>
       <c r="AR17" t="n">
-        <v>11.29</v>
+        <v>0.8</v>
       </c>
       <c r="AS17" t="n">
-        <v>0.89</v>
+        <v>0.46</v>
       </c>
       <c r="AT17" t="n">
-        <v>0.8</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AU17" t="n">
-        <v>0.46</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AV17" t="n">
-        <v>0.07000000000000001</v>
+        <v>2.57</v>
       </c>
       <c r="AW17" t="n">
-        <v>0.07000000000000001</v>
+        <v>3.37</v>
       </c>
       <c r="AX17" t="n">
-        <v>2.57</v>
+        <v>0.04</v>
       </c>
       <c r="AY17" t="n">
-        <v>3.37</v>
+        <v>0.01</v>
       </c>
       <c r="AZ17" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>18.32</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>303.97</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="BM17" t="n">
         <v>0.04</v>
       </c>
-      <c r="BA17" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="BB17" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="BC17" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="BD17" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="BE17" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="BF17" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="BG17" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>18.32</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>303.97</v>
-      </c>
-      <c r="BM17" t="n">
-        <v>19.57</v>
-      </c>
       <c r="BN17" t="n">
-        <v>0.66</v>
+        <v>96.87</v>
       </c>
       <c r="BO17" t="n">
-        <v>0.04</v>
+        <v>12.23</v>
       </c>
       <c r="BP17" t="n">
-        <v>96.87</v>
+        <v>2000</v>
       </c>
       <c r="BQ17" t="n">
-        <v>12.23</v>
+        <v>0</v>
       </c>
       <c r="BR17" t="n">
         <v>2000</v>
@@ -4331,22 +4331,22 @@
         <v>0</v>
       </c>
       <c r="BT17" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU17" t="n">
         <v>0</v>
       </c>
       <c r="BV17" t="n">
-        <v>15</v>
+        <v>0.72</v>
       </c>
       <c r="BW17" t="n">
         <v>0</v>
       </c>
       <c r="BX17" t="n">
-        <v>0.72</v>
+        <v>34.39</v>
       </c>
       <c r="BY17" t="n">
-        <v>0</v>
+        <v>1.95</v>
       </c>
       <c r="BZ17" t="n">
         <v>0.53</v>
@@ -4469,115 +4469,115 @@
       <c r="AE18" t="n">
         <v>241.41</v>
       </c>
-      <c r="AF18" t="n">
-        <v>35.38</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="n">
+        <v>592235.54</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>116.4</v>
+      </c>
       <c r="AJ18" t="n">
-        <v>592235.54</v>
+        <v>20</v>
       </c>
       <c r="AK18" t="n">
-        <v>116.4</v>
+        <v>0</v>
       </c>
       <c r="AL18" t="n">
-        <v>20</v>
+        <v>472.77</v>
       </c>
       <c r="AM18" t="n">
-        <v>0</v>
+        <v>38.37</v>
       </c>
       <c r="AN18" t="n">
-        <v>472.77</v>
+        <v>504.06</v>
       </c>
       <c r="AO18" t="n">
-        <v>38.37</v>
+        <v>14.01</v>
       </c>
       <c r="AP18" t="n">
-        <v>504.06</v>
+        <v>12.12</v>
       </c>
       <c r="AQ18" t="n">
-        <v>14.01</v>
+        <v>1.94</v>
       </c>
       <c r="AR18" t="n">
-        <v>12.12</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS18" t="n">
-        <v>1.94</v>
+        <v>0.53</v>
       </c>
       <c r="AT18" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="AU18" t="n">
-        <v>0.53</v>
+        <v>0.1</v>
       </c>
       <c r="AV18" t="n">
-        <v>0.06</v>
+        <v>2.36</v>
       </c>
       <c r="AW18" t="n">
-        <v>0.1</v>
+        <v>1.92</v>
       </c>
       <c r="AX18" t="n">
-        <v>2.36</v>
+        <v>0.04</v>
       </c>
       <c r="AY18" t="n">
-        <v>1.92</v>
+        <v>0.01</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0.04</v>
+        <v>3.57</v>
       </c>
       <c r="BA18" t="n">
-        <v>0.01</v>
+        <v>0.92</v>
       </c>
       <c r="BB18" t="n">
-        <v>3.57</v>
+        <v>1.67</v>
       </c>
       <c r="BC18" t="n">
-        <v>0.92</v>
+        <v>0.64</v>
       </c>
       <c r="BD18" t="n">
-        <v>1.67</v>
+        <v>0.05</v>
       </c>
       <c r="BE18" t="n">
-        <v>0.64</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="BF18" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>304.58</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>21.22</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="BM18" t="n">
         <v>0.05</v>
       </c>
-      <c r="BG18" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="BH18" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="BI18" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="BJ18" t="n">
-        <v>18.35</v>
-      </c>
-      <c r="BK18" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="BL18" t="n">
-        <v>304.58</v>
-      </c>
-      <c r="BM18" t="n">
-        <v>21.22</v>
-      </c>
       <c r="BN18" t="n">
-        <v>0.66</v>
+        <v>96.48</v>
       </c>
       <c r="BO18" t="n">
-        <v>0.05</v>
+        <v>13.26</v>
       </c>
       <c r="BP18" t="n">
-        <v>96.48</v>
+        <v>2000</v>
       </c>
       <c r="BQ18" t="n">
-        <v>13.26</v>
+        <v>0</v>
       </c>
       <c r="BR18" t="n">
         <v>2000</v>
@@ -4586,22 +4586,22 @@
         <v>0</v>
       </c>
       <c r="BT18" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU18" t="n">
         <v>0</v>
       </c>
       <c r="BV18" t="n">
-        <v>15</v>
+        <v>0.72</v>
       </c>
       <c r="BW18" t="n">
         <v>0</v>
       </c>
       <c r="BX18" t="n">
-        <v>0.72</v>
+        <v>35.38</v>
       </c>
       <c r="BY18" t="n">
-        <v>0</v>
+        <v>3.41</v>
       </c>
       <c r="BZ18" t="n">
         <v>0.53</v>
@@ -4724,115 +4724,115 @@
       <c r="AE19" t="n">
         <v>144.57</v>
       </c>
-      <c r="AF19" t="n">
-        <v>34.58</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="n">
+        <v>592200.27</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>117.12</v>
+      </c>
       <c r="AJ19" t="n">
-        <v>592200.27</v>
+        <v>20</v>
       </c>
       <c r="AK19" t="n">
-        <v>117.12</v>
+        <v>0</v>
       </c>
       <c r="AL19" t="n">
-        <v>20</v>
+        <v>467.3</v>
       </c>
       <c r="AM19" t="n">
-        <v>0</v>
+        <v>24.91</v>
       </c>
       <c r="AN19" t="n">
-        <v>467.3</v>
+        <v>499.05</v>
       </c>
       <c r="AO19" t="n">
-        <v>24.91</v>
+        <v>17.89</v>
       </c>
       <c r="AP19" t="n">
-        <v>499.05</v>
+        <v>10.39</v>
       </c>
       <c r="AQ19" t="n">
-        <v>17.89</v>
+        <v>2.92</v>
       </c>
       <c r="AR19" t="n">
-        <v>10.39</v>
+        <v>1.39</v>
       </c>
       <c r="AS19" t="n">
-        <v>2.92</v>
+        <v>0.82</v>
       </c>
       <c r="AT19" t="n">
-        <v>1.39</v>
+        <v>0.02</v>
       </c>
       <c r="AU19" t="n">
-        <v>0.82</v>
+        <v>0.02</v>
       </c>
       <c r="AV19" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AY19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AZ19" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="BC19" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="BD19" t="n">
         <v>0.02</v>
       </c>
-      <c r="AW19" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="AX19" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="AY19" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="AZ19" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="BA19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="BB19" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="BC19" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="BD19" t="n">
-        <v>1.57</v>
-      </c>
       <c r="BE19" t="n">
-        <v>0.47</v>
+        <v>0.04</v>
       </c>
       <c r="BF19" t="n">
-        <v>0.02</v>
+        <v>0.59</v>
       </c>
       <c r="BG19" t="n">
-        <v>0.04</v>
+        <v>0.26</v>
       </c>
       <c r="BH19" t="n">
-        <v>0.59</v>
+        <v>18.43</v>
       </c>
       <c r="BI19" t="n">
-        <v>0.26</v>
+        <v>0.73</v>
       </c>
       <c r="BJ19" t="n">
-        <v>18.43</v>
+        <v>306.12</v>
       </c>
       <c r="BK19" t="n">
-        <v>0.73</v>
+        <v>14.77</v>
       </c>
       <c r="BL19" t="n">
-        <v>306.12</v>
+        <v>0.67</v>
       </c>
       <c r="BM19" t="n">
-        <v>14.77</v>
+        <v>0.03</v>
       </c>
       <c r="BN19" t="n">
-        <v>0.67</v>
+        <v>95.52</v>
       </c>
       <c r="BO19" t="n">
-        <v>0.03</v>
+        <v>9.23</v>
       </c>
       <c r="BP19" t="n">
-        <v>95.52</v>
+        <v>2000</v>
       </c>
       <c r="BQ19" t="n">
-        <v>9.23</v>
+        <v>0</v>
       </c>
       <c r="BR19" t="n">
         <v>2000</v>
@@ -4841,22 +4841,22 @@
         <v>0</v>
       </c>
       <c r="BT19" t="n">
-        <v>2000</v>
+        <v>15</v>
       </c>
       <c r="BU19" t="n">
         <v>0</v>
       </c>
       <c r="BV19" t="n">
-        <v>15</v>
+        <v>0.72</v>
       </c>
       <c r="BW19" t="n">
         <v>0</v>
       </c>
       <c r="BX19" t="n">
-        <v>0.72</v>
+        <v>34.58</v>
       </c>
       <c r="BY19" t="n">
-        <v>0</v>
+        <v>4.01</v>
       </c>
       <c r="BZ19" t="n">
         <v>0.53</v>
@@ -4988,27 +4988,23 @@
         <v>423.28</v>
       </c>
       <c r="AF20" t="n">
-        <v>80.27</v>
+        <v>0.03</v>
       </c>
       <c r="AG20" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AI20" t="n">
         <v>0.02</v>
       </c>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
-      <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="inlineStr"/>
-      <c r="AN20" t="n">
+      <c r="AL20" t="n">
         <v>517.2</v>
       </c>
-      <c r="AO20" t="n">
+      <c r="AM20" t="n">
         <v>36.65</v>
       </c>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
       <c r="AP20" t="inlineStr"/>
       <c r="AQ20" t="inlineStr"/>
       <c r="AR20" t="inlineStr"/>
@@ -5027,55 +5023,59 @@
       <c r="BE20" t="inlineStr"/>
       <c r="BF20" t="inlineStr"/>
       <c r="BG20" t="inlineStr"/>
-      <c r="BH20" t="inlineStr"/>
-      <c r="BI20" t="inlineStr"/>
+      <c r="BH20" t="n">
+        <v>22.85</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>0.8</v>
+      </c>
       <c r="BJ20" t="n">
-        <v>22.85</v>
+        <v>395.99</v>
       </c>
       <c r="BK20" t="n">
-        <v>0.8</v>
+        <v>16.28</v>
       </c>
       <c r="BL20" t="n">
-        <v>395.99</v>
+        <v>0.86</v>
       </c>
       <c r="BM20" t="n">
-        <v>16.28</v>
+        <v>0.04</v>
       </c>
       <c r="BN20" t="n">
-        <v>0.86</v>
+        <v>39.35</v>
       </c>
       <c r="BO20" t="n">
-        <v>0.04</v>
+        <v>10.18</v>
       </c>
       <c r="BP20" t="n">
-        <v>39.35</v>
+        <v>2000</v>
       </c>
       <c r="BQ20" t="n">
-        <v>10.18</v>
+        <v>0</v>
       </c>
       <c r="BR20" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS20" t="n">
         <v>0</v>
       </c>
       <c r="BT20" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU20" t="n">
         <v>0</v>
       </c>
       <c r="BV20" t="n">
-        <v>19</v>
+        <v>0.79</v>
       </c>
       <c r="BW20" t="n">
         <v>0</v>
       </c>
       <c r="BX20" t="n">
-        <v>0.79</v>
+        <v>80.27</v>
       </c>
       <c r="BY20" t="n">
-        <v>0</v>
+        <v>8.75</v>
       </c>
       <c r="BZ20" t="n">
         <v>0.48</v>
@@ -5203,27 +5203,23 @@
         <v>393.07</v>
       </c>
       <c r="AF21" t="n">
-        <v>77.51000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AG21" t="n">
-        <v>15.42</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="AI21" t="n">
         <v>0.1</v>
       </c>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
-      <c r="AL21" t="inlineStr"/>
-      <c r="AM21" t="inlineStr"/>
-      <c r="AN21" t="n">
+      <c r="AL21" t="n">
         <v>567.65</v>
       </c>
-      <c r="AO21" t="n">
+      <c r="AM21" t="n">
         <v>103.37</v>
       </c>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
       <c r="AP21" t="inlineStr"/>
       <c r="AQ21" t="inlineStr"/>
       <c r="AR21" t="inlineStr"/>
@@ -5242,55 +5238,59 @@
       <c r="BE21" t="inlineStr"/>
       <c r="BF21" t="inlineStr"/>
       <c r="BG21" t="inlineStr"/>
-      <c r="BH21" t="inlineStr"/>
-      <c r="BI21" t="inlineStr"/>
+      <c r="BH21" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="BI21" t="n">
+        <v>1.93</v>
+      </c>
       <c r="BJ21" t="n">
-        <v>21.61</v>
+        <v>370.64</v>
       </c>
       <c r="BK21" t="n">
-        <v>1.93</v>
+        <v>39.1</v>
       </c>
       <c r="BL21" t="n">
-        <v>370.64</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="BM21" t="n">
-        <v>39.1</v>
+        <v>0.09</v>
       </c>
       <c r="BN21" t="n">
-        <v>0.8100000000000001</v>
+        <v>55.19</v>
       </c>
       <c r="BO21" t="n">
-        <v>0.09</v>
+        <v>24.44</v>
       </c>
       <c r="BP21" t="n">
-        <v>55.19</v>
+        <v>2000</v>
       </c>
       <c r="BQ21" t="n">
-        <v>24.44</v>
+        <v>0</v>
       </c>
       <c r="BR21" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS21" t="n">
         <v>0</v>
       </c>
       <c r="BT21" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU21" t="n">
         <v>0</v>
       </c>
       <c r="BV21" t="n">
-        <v>19</v>
+        <v>0.79</v>
       </c>
       <c r="BW21" t="n">
         <v>0</v>
       </c>
       <c r="BX21" t="n">
-        <v>0.79</v>
+        <v>77.51000000000001</v>
       </c>
       <c r="BY21" t="n">
-        <v>0</v>
+        <v>15.42</v>
       </c>
       <c r="BZ21" t="n">
         <v>0.43</v>
@@ -5418,27 +5418,23 @@
         <v>479.13</v>
       </c>
       <c r="AF22" t="n">
-        <v>101.47</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AG22" t="n">
-        <v>52.75</v>
-      </c>
-      <c r="AH22" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="AI22" t="n">
         <v>0.06</v>
       </c>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="n">
+      <c r="AL22" t="n">
         <v>498.3</v>
       </c>
-      <c r="AO22" t="n">
+      <c r="AM22" t="n">
         <v>49.19</v>
       </c>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
       <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
@@ -5457,55 +5453,59 @@
       <c r="BE22" t="inlineStr"/>
       <c r="BF22" t="inlineStr"/>
       <c r="BG22" t="inlineStr"/>
-      <c r="BH22" t="inlineStr"/>
-      <c r="BI22" t="inlineStr"/>
+      <c r="BH22" t="n">
+        <v>23.05</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>1.42</v>
+      </c>
       <c r="BJ22" t="n">
-        <v>23.05</v>
+        <v>399.94</v>
       </c>
       <c r="BK22" t="n">
-        <v>1.42</v>
+        <v>28.9</v>
       </c>
       <c r="BL22" t="n">
-        <v>399.94</v>
+        <v>0.87</v>
       </c>
       <c r="BM22" t="n">
-        <v>28.9</v>
+        <v>0.06</v>
       </c>
       <c r="BN22" t="n">
-        <v>0.87</v>
+        <v>36.88</v>
       </c>
       <c r="BO22" t="n">
-        <v>0.06</v>
+        <v>18.06</v>
       </c>
       <c r="BP22" t="n">
-        <v>36.88</v>
+        <v>2000</v>
       </c>
       <c r="BQ22" t="n">
-        <v>18.06</v>
+        <v>0</v>
       </c>
       <c r="BR22" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS22" t="n">
         <v>0</v>
       </c>
       <c r="BT22" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU22" t="n">
         <v>0</v>
       </c>
       <c r="BV22" t="n">
-        <v>19</v>
+        <v>0.79</v>
       </c>
       <c r="BW22" t="n">
         <v>0</v>
       </c>
       <c r="BX22" t="n">
-        <v>0.79</v>
+        <v>101.47</v>
       </c>
       <c r="BY22" t="n">
-        <v>0</v>
+        <v>52.75</v>
       </c>
       <c r="BZ22" t="n">
         <v>0.5</v>
@@ -5633,27 +5633,23 @@
         <v>289.8</v>
       </c>
       <c r="AF23" t="n">
-        <v>78.02</v>
+        <v>0.04</v>
       </c>
       <c r="AG23" t="n">
-        <v>10.48</v>
-      </c>
-      <c r="AH23" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AI23" t="n">
         <v>0.03</v>
       </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr"/>
-      <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="n">
+      <c r="AL23" t="n">
         <v>497.57</v>
       </c>
-      <c r="AO23" t="n">
+      <c r="AM23" t="n">
         <v>47.07</v>
       </c>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr"/>
       <c r="AR23" t="inlineStr"/>
@@ -5672,55 +5668,59 @@
       <c r="BE23" t="inlineStr"/>
       <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr"/>
-      <c r="BH23" t="inlineStr"/>
-      <c r="BI23" t="inlineStr"/>
+      <c r="BH23" t="n">
+        <v>22.55</v>
+      </c>
+      <c r="BI23" t="n">
+        <v>0.99</v>
+      </c>
       <c r="BJ23" t="n">
-        <v>22.55</v>
+        <v>389.88</v>
       </c>
       <c r="BK23" t="n">
-        <v>0.99</v>
+        <v>20.01</v>
       </c>
       <c r="BL23" t="n">
-        <v>389.88</v>
+        <v>0.85</v>
       </c>
       <c r="BM23" t="n">
-        <v>20.01</v>
+        <v>0.04</v>
       </c>
       <c r="BN23" t="n">
-        <v>0.85</v>
+        <v>43.17</v>
       </c>
       <c r="BO23" t="n">
-        <v>0.04</v>
+        <v>12.5</v>
       </c>
       <c r="BP23" t="n">
-        <v>43.17</v>
+        <v>2000</v>
       </c>
       <c r="BQ23" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="BR23" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="BS23" t="n">
         <v>0</v>
       </c>
       <c r="BT23" t="n">
-        <v>1000</v>
+        <v>19</v>
       </c>
       <c r="BU23" t="n">
         <v>0</v>
       </c>
       <c r="BV23" t="n">
-        <v>19</v>
+        <v>0.79</v>
       </c>
       <c r="BW23" t="n">
         <v>0</v>
       </c>
       <c r="BX23" t="n">
-        <v>0.79</v>
+        <v>78.02</v>
       </c>
       <c r="BY23" t="n">
-        <v>0</v>
+        <v>10.48</v>
       </c>
       <c r="BZ23" t="n">
         <v>0.5</v>
@@ -5852,27 +5852,23 @@
         <v>4.07</v>
       </c>
       <c r="AF24" t="n">
-        <v>70.09999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="AG24" t="n">
-        <v>5.89</v>
-      </c>
-      <c r="AH24" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="AI24" t="n">
         <v>0.01</v>
       </c>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="n">
+      <c r="AL24" t="n">
         <v>458.37</v>
       </c>
-      <c r="AO24" t="n">
+      <c r="AM24" t="n">
         <v>24.12</v>
       </c>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
       <c r="AP24" t="inlineStr"/>
       <c r="AQ24" t="inlineStr"/>
       <c r="AR24" t="inlineStr"/>
@@ -5891,55 +5887,59 @@
       <c r="BE24" t="inlineStr"/>
       <c r="BF24" t="inlineStr"/>
       <c r="BG24" t="inlineStr"/>
-      <c r="BH24" t="inlineStr"/>
-      <c r="BI24" t="inlineStr"/>
+      <c r="BH24" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="BI24" t="n">
+        <v>0.28</v>
+      </c>
       <c r="BJ24" t="n">
-        <v>18.8</v>
+        <v>313.67</v>
       </c>
       <c r="BK24" t="n">
-        <v>0.28</v>
+        <v>5.73</v>
       </c>
       <c r="BL24" t="n">
-        <v>313.67</v>
+        <v>0.68</v>
       </c>
       <c r="BM24" t="n">
-        <v>5.73</v>
+        <v>0.01</v>
       </c>
       <c r="BN24" t="n">
-        <v>0.68</v>
+        <v>90.8</v>
       </c>
       <c r="BO24" t="n">
-        <v>0.01</v>
+        <v>3.58</v>
       </c>
       <c r="BP24" t="n">
-        <v>90.8</v>
+        <v>4500</v>
       </c>
       <c r="BQ24" t="n">
-        <v>3.58</v>
+        <v>0</v>
       </c>
       <c r="BR24" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS24" t="n">
         <v>0</v>
       </c>
       <c r="BT24" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU24" t="n">
         <v>0</v>
       </c>
       <c r="BV24" t="n">
-        <v>10</v>
+        <v>0.54</v>
       </c>
       <c r="BW24" t="n">
         <v>0</v>
       </c>
       <c r="BX24" t="n">
-        <v>0.54</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="BY24" t="n">
-        <v>0</v>
+        <v>5.89</v>
       </c>
       <c r="BZ24" t="n">
         <v>0.54</v>
@@ -6067,27 +6067,23 @@
         <v>12.72</v>
       </c>
       <c r="AF25" t="n">
-        <v>69.55</v>
+        <v>0.02</v>
       </c>
       <c r="AG25" t="n">
-        <v>9.630000000000001</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="AI25" t="n">
         <v>0.01</v>
       </c>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
-      <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="n">
+      <c r="AL25" t="n">
         <v>484.91</v>
       </c>
-      <c r="AO25" t="n">
+      <c r="AM25" t="n">
         <v>63.86</v>
       </c>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
       <c r="AP25" t="inlineStr"/>
       <c r="AQ25" t="inlineStr"/>
       <c r="AR25" t="inlineStr"/>
@@ -6106,55 +6102,59 @@
       <c r="BE25" t="inlineStr"/>
       <c r="BF25" t="inlineStr"/>
       <c r="BG25" t="inlineStr"/>
-      <c r="BH25" t="inlineStr"/>
-      <c r="BI25" t="inlineStr"/>
+      <c r="BH25" t="n">
+        <v>19.17</v>
+      </c>
+      <c r="BI25" t="n">
+        <v>0.9399999999999999</v>
+      </c>
       <c r="BJ25" t="n">
-        <v>19.17</v>
+        <v>321.26</v>
       </c>
       <c r="BK25" t="n">
-        <v>0.9399999999999999</v>
+        <v>19.08</v>
       </c>
       <c r="BL25" t="n">
-        <v>321.26</v>
+        <v>0.7</v>
       </c>
       <c r="BM25" t="n">
-        <v>19.08</v>
+        <v>0.04</v>
       </c>
       <c r="BN25" t="n">
-        <v>0.7</v>
+        <v>86.06</v>
       </c>
       <c r="BO25" t="n">
-        <v>0.04</v>
+        <v>11.93</v>
       </c>
       <c r="BP25" t="n">
-        <v>86.06</v>
+        <v>4500</v>
       </c>
       <c r="BQ25" t="n">
-        <v>11.93</v>
+        <v>0</v>
       </c>
       <c r="BR25" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS25" t="n">
         <v>0</v>
       </c>
       <c r="BT25" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU25" t="n">
         <v>0</v>
       </c>
       <c r="BV25" t="n">
-        <v>10</v>
+        <v>0.54</v>
       </c>
       <c r="BW25" t="n">
         <v>0</v>
       </c>
       <c r="BX25" t="n">
-        <v>0.54</v>
+        <v>69.55</v>
       </c>
       <c r="BY25" t="n">
-        <v>0</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="BZ25" t="n">
         <v>0.52</v>
@@ -6282,27 +6282,23 @@
         <v>3.7</v>
       </c>
       <c r="AF26" t="n">
-        <v>72.20999999999999</v>
+        <v>0.02</v>
       </c>
       <c r="AG26" t="n">
-        <v>6.39</v>
-      </c>
-      <c r="AH26" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="AI26" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
       <c r="AJ26" t="inlineStr"/>
       <c r="AK26" t="inlineStr"/>
-      <c r="AL26" t="inlineStr"/>
-      <c r="AM26" t="inlineStr"/>
-      <c r="AN26" t="n">
+      <c r="AL26" t="n">
         <v>447.24</v>
       </c>
-      <c r="AO26" t="n">
+      <c r="AM26" t="n">
         <v>11.29</v>
       </c>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
       <c r="AP26" t="inlineStr"/>
       <c r="AQ26" t="inlineStr"/>
       <c r="AR26" t="inlineStr"/>
@@ -6321,55 +6317,59 @@
       <c r="BE26" t="inlineStr"/>
       <c r="BF26" t="inlineStr"/>
       <c r="BG26" t="inlineStr"/>
-      <c r="BH26" t="inlineStr"/>
-      <c r="BI26" t="inlineStr"/>
+      <c r="BH26" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="BI26" t="n">
+        <v>0.83</v>
+      </c>
       <c r="BJ26" t="n">
-        <v>20.2</v>
+        <v>342.02</v>
       </c>
       <c r="BK26" t="n">
-        <v>0.83</v>
+        <v>16.9</v>
       </c>
       <c r="BL26" t="n">
-        <v>342.02</v>
+        <v>0.75</v>
       </c>
       <c r="BM26" t="n">
-        <v>16.9</v>
+        <v>0.04</v>
       </c>
       <c r="BN26" t="n">
-        <v>0.75</v>
+        <v>73.08</v>
       </c>
       <c r="BO26" t="n">
-        <v>0.04</v>
+        <v>10.56</v>
       </c>
       <c r="BP26" t="n">
-        <v>73.08</v>
+        <v>4500</v>
       </c>
       <c r="BQ26" t="n">
-        <v>10.56</v>
+        <v>0</v>
       </c>
       <c r="BR26" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS26" t="n">
         <v>0</v>
       </c>
       <c r="BT26" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU26" t="n">
         <v>0</v>
       </c>
       <c r="BV26" t="n">
-        <v>10</v>
+        <v>0.54</v>
       </c>
       <c r="BW26" t="n">
         <v>0</v>
       </c>
       <c r="BX26" t="n">
-        <v>0.54</v>
+        <v>72.20999999999999</v>
       </c>
       <c r="BY26" t="n">
-        <v>0</v>
+        <v>6.39</v>
       </c>
       <c r="BZ26" t="n">
         <v>0.55</v>
@@ -6497,27 +6497,23 @@
         <v>2.13</v>
       </c>
       <c r="AF27" t="n">
-        <v>72.58</v>
+        <v>0.02</v>
       </c>
       <c r="AG27" t="n">
-        <v>4.07</v>
-      </c>
-      <c r="AH27" t="n">
         <v>0.02</v>
       </c>
-      <c r="AI27" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-      <c r="AL27" t="inlineStr"/>
-      <c r="AM27" t="inlineStr"/>
-      <c r="AN27" t="n">
+      <c r="AL27" t="n">
         <v>450.2</v>
       </c>
-      <c r="AO27" t="n">
+      <c r="AM27" t="n">
         <v>29.2</v>
       </c>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
       <c r="AP27" t="inlineStr"/>
       <c r="AQ27" t="inlineStr"/>
       <c r="AR27" t="inlineStr"/>
@@ -6536,55 +6532,59 @@
       <c r="BE27" t="inlineStr"/>
       <c r="BF27" t="inlineStr"/>
       <c r="BG27" t="inlineStr"/>
-      <c r="BH27" t="inlineStr"/>
-      <c r="BI27" t="inlineStr"/>
+      <c r="BH27" t="n">
+        <v>19.51</v>
+      </c>
+      <c r="BI27" t="n">
+        <v>1.18</v>
+      </c>
       <c r="BJ27" t="n">
-        <v>19.51</v>
+        <v>328.17</v>
       </c>
       <c r="BK27" t="n">
-        <v>1.18</v>
+        <v>24.05</v>
       </c>
       <c r="BL27" t="n">
-        <v>328.17</v>
+        <v>0.72</v>
       </c>
       <c r="BM27" t="n">
-        <v>24.05</v>
+        <v>0.05</v>
       </c>
       <c r="BN27" t="n">
-        <v>0.72</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="BO27" t="n">
-        <v>0.05</v>
+        <v>15.03</v>
       </c>
       <c r="BP27" t="n">
-        <v>81.73999999999999</v>
+        <v>4500</v>
       </c>
       <c r="BQ27" t="n">
-        <v>15.03</v>
+        <v>0</v>
       </c>
       <c r="BR27" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="BS27" t="n">
         <v>0</v>
       </c>
       <c r="BT27" t="n">
-        <v>3000</v>
+        <v>10</v>
       </c>
       <c r="BU27" t="n">
         <v>0</v>
       </c>
       <c r="BV27" t="n">
-        <v>10</v>
+        <v>0.54</v>
       </c>
       <c r="BW27" t="n">
         <v>0</v>
       </c>
       <c r="BX27" t="n">
-        <v>0.54</v>
+        <v>72.58</v>
       </c>
       <c r="BY27" t="n">
-        <v>0</v>
+        <v>4.07</v>
       </c>
       <c r="BZ27" t="n">
         <v>0.55</v>

</xml_diff>

<commit_message>
edit dummies colors revisando SLA
</commit_message>
<xml_diff>
--- a/Summary.xlsx
+++ b/Summary.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL27"/>
+  <dimension ref="A1:CP27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -736,6 +736,18 @@
         </is>
       </c>
       <c r="CL1" s="1" t="n"/>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="n"/>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="1" t="inlineStr"/>
@@ -1179,6 +1191,26 @@
           <t>std</t>
         </is>
       </c>
+      <c r="CM2" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="CN2" s="1" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="CO2" s="1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="CP2" s="1" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1459,6 +1491,18 @@
       <c r="CL4" t="n">
         <v>1.57</v>
       </c>
+      <c r="CM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n"/>
@@ -1723,6 +1767,18 @@
       <c r="CL5" t="n">
         <v>2.09</v>
       </c>
+      <c r="CM5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n"/>
@@ -1987,6 +2043,18 @@
       <c r="CL6" t="n">
         <v>1.15</v>
       </c>
+      <c r="CM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n"/>
@@ -2250,6 +2318,18 @@
       </c>
       <c r="CL7" t="n">
         <v>1.51</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2478,6 +2558,18 @@
       </c>
       <c r="CL8" t="n">
         <v>0.41</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2639,6 +2731,14 @@
         <v>3.99</v>
       </c>
       <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
@@ -2863,6 +2963,18 @@
       <c r="CL10" t="n">
         <v>0.43</v>
       </c>
+      <c r="CM10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n"/>
@@ -3087,6 +3199,18 @@
       <c r="CL11" t="n">
         <v>0.24</v>
       </c>
+      <c r="CM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -3315,6 +3439,18 @@
       <c r="CL12" t="n">
         <v>1.65</v>
       </c>
+      <c r="CM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
@@ -3539,6 +3675,18 @@
       <c r="CL13" t="n">
         <v>0.8100000000000001</v>
       </c>
+      <c r="CM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>
@@ -3763,6 +3911,18 @@
       <c r="CL14" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="CM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
@@ -3987,6 +4147,18 @@
       <c r="CL15" t="n">
         <v>1</v>
       </c>
+      <c r="CM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -4255,6 +4427,18 @@
       <c r="CL16" t="n">
         <v>1.47</v>
       </c>
+      <c r="CM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -4519,6 +4703,18 @@
       <c r="CL17" t="n">
         <v>0.76</v>
       </c>
+      <c r="CM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -4783,6 +4979,18 @@
       <c r="CL18" t="n">
         <v>1.3</v>
       </c>
+      <c r="CM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO18" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -5046,6 +5254,18 @@
       </c>
       <c r="CL19" t="n">
         <v>1.88</v>
+      </c>
+      <c r="CM19" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO19" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -5275,6 +5495,18 @@
       <c r="CL20" t="n">
         <v>0.74</v>
       </c>
+      <c r="CM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
@@ -5499,6 +5731,18 @@
       <c r="CL21" t="n">
         <v>1.18</v>
       </c>
+      <c r="CM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
@@ -5723,6 +5967,18 @@
       <c r="CL22" t="n">
         <v>0.66</v>
       </c>
+      <c r="CM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
@@ -5947,6 +6203,18 @@
       <c r="CL23" t="n">
         <v>0.9399999999999999</v>
       </c>
+      <c r="CM23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO23" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -6175,6 +6443,18 @@
       <c r="CL24" t="n">
         <v>0.5</v>
       </c>
+      <c r="CM24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
@@ -6399,6 +6679,18 @@
       <c r="CL25" t="n">
         <v>0.96</v>
       </c>
+      <c r="CM25" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
@@ -6623,6 +6915,18 @@
       <c r="CL26" t="n">
         <v>0.44</v>
       </c>
+      <c r="CM26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
@@ -6847,9 +7151,21 @@
       <c r="CL27" t="n">
         <v>0.37</v>
       </c>
+      <c r="CM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO27" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP27" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="52">
     <mergeCell ref="BY1:BZ1"/>
     <mergeCell ref="AG1:AH1"/>
     <mergeCell ref="AI1:AJ1"/>
@@ -6861,6 +7177,7 @@
     <mergeCell ref="AU1:AV1"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="CC1:CD1"/>
+    <mergeCell ref="CO1:CP1"/>
     <mergeCell ref="A16:A19"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
@@ -6884,6 +7201,7 @@
     <mergeCell ref="A20:A23"/>
     <mergeCell ref="AO1:AP1"/>
     <mergeCell ref="AE1:AF1"/>
+    <mergeCell ref="CM1:CN1"/>
     <mergeCell ref="AQ1:AR1"/>
     <mergeCell ref="AW1:AX1"/>
     <mergeCell ref="CE1:CF1"/>

</xml_diff>

<commit_message>
editado el cleaning para eliminar outliers.
</commit_message>
<xml_diff>
--- a/Summary.xlsx
+++ b/Summary.xlsx
@@ -758,10 +758,10 @@
         <v>14.05</v>
       </c>
       <c r="L6" t="n">
-        <v>23.08</v>
+        <v>23.65</v>
       </c>
       <c r="M6" t="n">
-        <v>1.19</v>
+        <v>1.5</v>
       </c>
       <c r="N6" t="n">
         <v>1.15</v>
@@ -770,16 +770,16 @@
         <v>0.14</v>
       </c>
       <c r="P6" t="n">
-        <v>20.2</v>
+        <v>20.83</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.97</v>
+        <v>3.48</v>
       </c>
       <c r="R6" t="n">
-        <v>18.89</v>
+        <v>18.28</v>
       </c>
       <c r="S6" t="n">
-        <v>1.51</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="7">
@@ -870,10 +870,10 @@
         <v>8.75</v>
       </c>
       <c r="J8" t="n">
-        <v>480.48</v>
+        <v>478</v>
       </c>
       <c r="K8" t="n">
-        <v>28.38</v>
+        <v>5.31</v>
       </c>
       <c r="L8" t="n">
         <v>15.29</v>
@@ -915,10 +915,10 @@
         <v>0.87</v>
       </c>
       <c r="F9" t="n">
-        <v>88.72</v>
+        <v>99.8</v>
       </c>
       <c r="G9" t="n">
-        <v>10.65</v>
+        <v>22.43</v>
       </c>
       <c r="H9" t="n">
         <v>78.19</v>
@@ -927,10 +927,10 @@
         <v>14.39</v>
       </c>
       <c r="J9" t="n">
-        <v>476.52</v>
+        <v>480.5</v>
       </c>
       <c r="K9" t="n">
-        <v>13.88</v>
+        <v>6.22</v>
       </c>
       <c r="L9" t="n">
         <v>15.69</v>
@@ -1218,10 +1218,10 @@
         <v>3.27</v>
       </c>
       <c r="J14" t="n">
-        <v>481.32</v>
+        <v>490.56</v>
       </c>
       <c r="K14" t="n">
-        <v>27.85</v>
+        <v>10.44</v>
       </c>
       <c r="L14" t="n">
         <v>12.04</v>
@@ -1275,10 +1275,10 @@
         <v>5.12</v>
       </c>
       <c r="J15" t="n">
-        <v>485.14</v>
+        <v>486.93</v>
       </c>
       <c r="K15" t="n">
-        <v>8.49</v>
+        <v>5.09</v>
       </c>
       <c r="L15" t="n">
         <v>11.1</v>
@@ -1287,10 +1287,10 @@
         <v>1.37</v>
       </c>
       <c r="N15" t="n">
-        <v>1.41</v>
+        <v>1.24</v>
       </c>
       <c r="O15" t="n">
-        <v>0.7</v>
+        <v>0.28</v>
       </c>
       <c r="P15" t="n">
         <v>8.94</v>
@@ -1342,10 +1342,10 @@
         <v>9.44</v>
       </c>
       <c r="L16" t="n">
-        <v>10.2</v>
+        <v>8.82</v>
       </c>
       <c r="M16" t="n">
-        <v>5.48</v>
+        <v>1.17</v>
       </c>
       <c r="N16" t="n">
         <v>0.43</v>
@@ -1753,10 +1753,10 @@
         <v>1.54</v>
       </c>
       <c r="N23" t="n">
-        <v>1.6</v>
+        <v>1.42</v>
       </c>
       <c r="O23" t="n">
-        <v>0.64</v>
+        <v>0.44</v>
       </c>
       <c r="P23" t="n">
         <v>11.12</v>

</xml_diff>